<commit_message>
feat: migracao completa para o supabase e integracao de paginas
</commit_message>
<xml_diff>
--- a/modelo_importacao_alunos.xlsx
+++ b/modelo_importacao_alunos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -477,124 +477,9 @@
           <t>senha</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Lucas Silva</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>111.222.333-44</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2010-05-15</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Manhã</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>3º Ano A</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>lucas.silva@aluno.seduc.pa.gov.br</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Mãe</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Maria Silva</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>(91) 99999-8888</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>senha@123</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Julia Souza</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>555.666.777-88</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2012-08-20</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Tarde</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2º Ano B</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>julia.souza@aluno.seduc.pa.gov.br</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Pai</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Carlos Souza</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>(91) 98888-7777</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Rota 02</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>senha@456</t>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>aeeAtendido</t>
         </is>
       </c>
     </row>

</xml_diff>